<commit_message>
Main Excel Project Workbook
</commit_message>
<xml_diff>
--- a/Operations Data Validation Dashboard.xlsx
+++ b/Operations Data Validation Dashboard.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
+  <workbookPr filterPrivacy="1" hidePivotFieldList="1" defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="108" windowWidth="14808" windowHeight="8016" firstSheet="3" activeTab="4"/>
+    <workbookView xWindow="240" yWindow="108" windowWidth="14808" windowHeight="8016" firstSheet="2" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="Operations Data" sheetId="2" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="797" uniqueCount="172">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="801" uniqueCount="173">
   <si>
     <t>Reference ID</t>
   </si>
@@ -508,9 +508,6 @@
     <t>Overall Validation</t>
   </si>
   <si>
-    <t>CompletionRate</t>
-  </si>
-  <si>
     <t>Items Category</t>
   </si>
   <si>
@@ -542,6 +539,12 @@
   </si>
   <si>
     <t>Operations Data Validation &amp; Performance Dashboard</t>
+  </si>
+  <si>
+    <t>Total Quantity</t>
+  </si>
+  <si>
+    <t>Avg. Quantity / Operation</t>
   </si>
 </sst>
 </file>
@@ -603,7 +606,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -644,12 +647,40 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color theme="1"/>
+      </left>
+      <right style="thin">
+        <color theme="1"/>
+      </right>
+      <top style="thin">
+        <color theme="1"/>
+      </top>
+      <bottom style="thin">
+        <color theme="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -664,9 +695,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -719,12 +747,620 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
-  <dxfs count="100">
+  <dxfs count="183">
+    <dxf>
+      <alignment horizontal="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" indent="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" indent="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" indent="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" indent="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <border>
+        <left/>
+        <right/>
+        <top/>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left/>
+        <right/>
+        <top/>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left/>
+        <right/>
+        <top/>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left/>
+        <right/>
+        <top/>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left/>
+        <right/>
+        <top/>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left/>
+        <right/>
+        <top/>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left/>
+        <right/>
+        <top/>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <right style="thin">
+          <color theme="1"/>
+        </right>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <right style="thin">
+          <color theme="1"/>
+        </right>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <right style="thin">
+          <color theme="1"/>
+        </right>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <right style="thin">
+          <color theme="1"/>
+        </right>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <right style="thin">
+          <color theme="1"/>
+        </right>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <right style="thin">
+          <color theme="1"/>
+        </right>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <right style="thin">
+          <color theme="1"/>
+        </right>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" indent="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" indent="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <border>
+        <left/>
+        <right/>
+        <top/>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left/>
+        <right/>
+        <top/>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left/>
+        <right/>
+        <top/>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left/>
+        <right/>
+        <top/>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left/>
+        <right/>
+        <top/>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left/>
+        <right/>
+        <top/>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" readingOrder="0"/>
+    </dxf>
     <dxf>
       <alignment horizontal="center" readingOrder="0"/>
     </dxf>
@@ -1404,676 +2040,7 @@
     </mc:Fallback>
   </mc:AlternateContent>
   <c:pivotSource>
-    <c:name>[Operations Data Validation Dashboard.xlsx]Operations Data Analysis!PivotTable1</c:name>
-    <c:fmtId val="14"/>
-  </c:pivotSource>
-  <c:chart>
-    <c:title>
-      <c:tx>
-        <c:rich>
-          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
-                <a:solidFill>
-                  <a:schemeClr val="tx1">
-                    <a:lumMod val="65000"/>
-                    <a:lumOff val="35000"/>
-                  </a:schemeClr>
-                </a:solidFill>
-                <a:latin typeface="+mn-lt"/>
-                <a:ea typeface="+mn-ea"/>
-                <a:cs typeface="+mn-cs"/>
-              </a:defRPr>
-            </a:pPr>
-            <a:r>
-              <a:rPr lang="en-IN" sz="1400" b="1" i="0" u="none" strike="noStrike" baseline="0">
-                <a:solidFill>
-                  <a:schemeClr val="tx1"/>
-                </a:solidFill>
-              </a:rPr>
-              <a:t>Operations Status by Department</a:t>
-            </a:r>
-            <a:endParaRPr lang="en-IN" b="1">
-              <a:solidFill>
-                <a:schemeClr val="tx1"/>
-              </a:solidFill>
-            </a:endParaRPr>
-          </a:p>
-        </c:rich>
-      </c:tx>
-      <c:layout>
-        <c:manualLayout>
-          <c:xMode val="edge"/>
-          <c:yMode val="edge"/>
-          <c:x val="0.22104855643044616"/>
-          <c:y val="2.7777777777777776E-2"/>
-        </c:manualLayout>
-      </c:layout>
-      <c:overlay val="0"/>
-      <c:spPr>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:effectLst/>
-      </c:spPr>
-      <c:txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr>
-            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="65000"/>
-                  <a:lumOff val="35000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:pPr>
-          <a:endParaRPr lang="en-US"/>
-        </a:p>
-      </c:txPr>
-    </c:title>
-    <c:autoTitleDeleted val="0"/>
-    <c:pivotFmts>
-      <c:pivotFmt>
-        <c:idx val="0"/>
-        <c:spPr>
-          <a:solidFill>
-            <a:schemeClr val="accent1"/>
-          </a:solidFill>
-          <a:ln>
-            <a:noFill/>
-          </a:ln>
-          <a:effectLst/>
-        </c:spPr>
-        <c:marker>
-          <c:symbol val="none"/>
-        </c:marker>
-      </c:pivotFmt>
-      <c:pivotFmt>
-        <c:idx val="1"/>
-        <c:spPr>
-          <a:solidFill>
-            <a:schemeClr val="accent1"/>
-          </a:solidFill>
-          <a:ln>
-            <a:noFill/>
-          </a:ln>
-          <a:effectLst/>
-        </c:spPr>
-        <c:marker>
-          <c:symbol val="none"/>
-        </c:marker>
-      </c:pivotFmt>
-      <c:pivotFmt>
-        <c:idx val="2"/>
-        <c:spPr>
-          <a:solidFill>
-            <a:schemeClr val="accent1"/>
-          </a:solidFill>
-          <a:ln>
-            <a:noFill/>
-          </a:ln>
-          <a:effectLst/>
-        </c:spPr>
-        <c:marker>
-          <c:symbol val="none"/>
-        </c:marker>
-        <c:dLbl>
-          <c:idx val="0"/>
-          <c:layout/>
-          <c:spPr>
-            <a:noFill/>
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:txPr>
-            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
-              <a:spAutoFit/>
-            </a:bodyPr>
-            <a:lstStyle/>
-            <a:p>
-              <a:pPr>
-                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1">
-                      <a:lumMod val="75000"/>
-                      <a:lumOff val="25000"/>
-                    </a:schemeClr>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:pPr>
-              <a:endParaRPr lang="en-US"/>
-            </a:p>
-          </c:txPr>
-          <c:dLblPos val="inEnd"/>
-          <c:showLegendKey val="0"/>
-          <c:showVal val="1"/>
-          <c:showCatName val="0"/>
-          <c:showSerName val="0"/>
-          <c:showPercent val="0"/>
-          <c:showBubbleSize val="0"/>
-          <c:extLst>
-            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
-              <c15:layout/>
-            </c:ext>
-          </c:extLst>
-        </c:dLbl>
-      </c:pivotFmt>
-    </c:pivotFmts>
-    <c:plotArea>
-      <c:layout>
-        <c:manualLayout>
-          <c:layoutTarget val="inner"/>
-          <c:xMode val="edge"/>
-          <c:yMode val="edge"/>
-          <c:x val="6.1176962374343329E-2"/>
-          <c:y val="0.15570948782535685"/>
-          <c:w val="0.76947221183875747"/>
-          <c:h val="0.74270248649649273"/>
-        </c:manualLayout>
-      </c:layout>
-      <c:barChart>
-        <c:barDir val="col"/>
-        <c:grouping val="clustered"/>
-        <c:varyColors val="0"/>
-        <c:ser>
-          <c:idx val="0"/>
-          <c:order val="0"/>
-          <c:tx>
-            <c:strRef>
-              <c:f>'Operations Data Analysis'!$B$3:$B$4</c:f>
-              <c:strCache>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>Completed</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:tx>
-          <c:spPr>
-            <a:solidFill>
-              <a:schemeClr val="accent1"/>
-            </a:solidFill>
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:invertIfNegative val="0"/>
-          <c:cat>
-            <c:strRef>
-              <c:f>'Operations Data Analysis'!$A$5:$A$9</c:f>
-              <c:strCache>
-                <c:ptCount val="4"/>
-                <c:pt idx="0">
-                  <c:v>Maintenance</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>Operations</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>Quality</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>Supply Chain</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>'Operations Data Analysis'!$B$5:$B$9</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="4"/>
-                <c:pt idx="0">
-                  <c:v>6</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>26</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>15</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>18</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:val>
-        </c:ser>
-        <c:ser>
-          <c:idx val="1"/>
-          <c:order val="1"/>
-          <c:tx>
-            <c:strRef>
-              <c:f>'Operations Data Analysis'!$C$3:$C$4</c:f>
-              <c:strCache>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>Pending</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:tx>
-          <c:spPr>
-            <a:solidFill>
-              <a:schemeClr val="accent2"/>
-            </a:solidFill>
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:invertIfNegative val="0"/>
-          <c:cat>
-            <c:strRef>
-              <c:f>'Operations Data Analysis'!$A$5:$A$9</c:f>
-              <c:strCache>
-                <c:ptCount val="4"/>
-                <c:pt idx="0">
-                  <c:v>Maintenance</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>Operations</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>Quality</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>Supply Chain</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>'Operations Data Analysis'!$C$5:$C$9</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="4"/>
-                <c:pt idx="0">
-                  <c:v>2</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>1</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>2</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>2</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:val>
-        </c:ser>
-        <c:ser>
-          <c:idx val="2"/>
-          <c:order val="2"/>
-          <c:tx>
-            <c:strRef>
-              <c:f>'Operations Data Analysis'!$D$3:$D$4</c:f>
-              <c:strCache>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>In Progress</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:tx>
-          <c:spPr>
-            <a:solidFill>
-              <a:schemeClr val="accent3"/>
-            </a:solidFill>
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:invertIfNegative val="0"/>
-          <c:dLbls>
-            <c:spPr>
-              <a:noFill/>
-              <a:ln>
-                <a:noFill/>
-              </a:ln>
-              <a:effectLst/>
-            </c:spPr>
-            <c:txPr>
-              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
-                <a:spAutoFit/>
-              </a:bodyPr>
-              <a:lstStyle/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                    <a:solidFill>
-                      <a:schemeClr val="tx1">
-                        <a:lumMod val="75000"/>
-                        <a:lumOff val="25000"/>
-                      </a:schemeClr>
-                    </a:solidFill>
-                    <a:latin typeface="+mn-lt"/>
-                    <a:ea typeface="+mn-ea"/>
-                    <a:cs typeface="+mn-cs"/>
-                  </a:defRPr>
-                </a:pPr>
-                <a:endParaRPr lang="en-US"/>
-              </a:p>
-            </c:txPr>
-            <c:dLblPos val="inEnd"/>
-            <c:showLegendKey val="0"/>
-            <c:showVal val="1"/>
-            <c:showCatName val="0"/>
-            <c:showSerName val="0"/>
-            <c:showPercent val="0"/>
-            <c:showBubbleSize val="0"/>
-            <c:showLeaderLines val="0"/>
-            <c:extLst>
-              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
-                <c15:layout/>
-                <c15:showLeaderLines val="1"/>
-                <c15:leaderLines>
-                  <c:spPr>
-                    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-                      <a:solidFill>
-                        <a:schemeClr val="tx1">
-                          <a:lumMod val="35000"/>
-                          <a:lumOff val="65000"/>
-                        </a:schemeClr>
-                      </a:solidFill>
-                      <a:round/>
-                    </a:ln>
-                    <a:effectLst/>
-                  </c:spPr>
-                </c15:leaderLines>
-              </c:ext>
-            </c:extLst>
-          </c:dLbls>
-          <c:cat>
-            <c:strRef>
-              <c:f>'Operations Data Analysis'!$A$5:$A$9</c:f>
-              <c:strCache>
-                <c:ptCount val="4"/>
-                <c:pt idx="0">
-                  <c:v>Maintenance</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>Operations</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>Quality</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>Supply Chain</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>'Operations Data Analysis'!$D$5:$D$9</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="4"/>
-                <c:pt idx="0">
-                  <c:v>1</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>2</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>5</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:val>
-        </c:ser>
-        <c:dLbls>
-          <c:showLegendKey val="0"/>
-          <c:showVal val="0"/>
-          <c:showCatName val="0"/>
-          <c:showSerName val="0"/>
-          <c:showPercent val="0"/>
-          <c:showBubbleSize val="0"/>
-        </c:dLbls>
-        <c:gapWidth val="75"/>
-        <c:overlap val="40"/>
-        <c:axId val="-1537117440"/>
-        <c:axId val="-1537121792"/>
-      </c:barChart>
-      <c:catAx>
-        <c:axId val="-1537117440"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-        </c:scaling>
-        <c:delete val="0"/>
-        <c:axPos val="b"/>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
-        <c:majorTickMark val="none"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
-        <c:spPr>
-          <a:noFill/>
-          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-            <a:solidFill>
-              <a:schemeClr val="tx1">
-                <a:lumMod val="15000"/>
-                <a:lumOff val="85000"/>
-              </a:schemeClr>
-            </a:solidFill>
-            <a:round/>
-          </a:ln>
-          <a:effectLst/>
-        </c:spPr>
-        <c:txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                <a:solidFill>
-                  <a:schemeClr val="tx1">
-                    <a:lumMod val="65000"/>
-                    <a:lumOff val="35000"/>
-                  </a:schemeClr>
-                </a:solidFill>
-                <a:latin typeface="+mn-lt"/>
-                <a:ea typeface="+mn-ea"/>
-                <a:cs typeface="+mn-cs"/>
-              </a:defRPr>
-            </a:pPr>
-            <a:endParaRPr lang="en-US"/>
-          </a:p>
-        </c:txPr>
-        <c:crossAx val="-1537121792"/>
-        <c:crosses val="autoZero"/>
-        <c:auto val="1"/>
-        <c:lblAlgn val="ctr"/>
-        <c:lblOffset val="100"/>
-        <c:noMultiLvlLbl val="0"/>
-      </c:catAx>
-      <c:valAx>
-        <c:axId val="-1537121792"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-        </c:scaling>
-        <c:delete val="0"/>
-        <c:axPos val="l"/>
-        <c:majorGridlines>
-          <c:spPr>
-            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="15000"/>
-                  <a:lumOff val="85000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-        </c:majorGridlines>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
-        <c:majorTickMark val="none"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
-        <c:spPr>
-          <a:noFill/>
-          <a:ln>
-            <a:noFill/>
-          </a:ln>
-          <a:effectLst/>
-        </c:spPr>
-        <c:txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                <a:solidFill>
-                  <a:schemeClr val="tx1">
-                    <a:lumMod val="65000"/>
-                    <a:lumOff val="35000"/>
-                  </a:schemeClr>
-                </a:solidFill>
-                <a:latin typeface="+mn-lt"/>
-                <a:ea typeface="+mn-ea"/>
-                <a:cs typeface="+mn-cs"/>
-              </a:defRPr>
-            </a:pPr>
-            <a:endParaRPr lang="en-US"/>
-          </a:p>
-        </c:txPr>
-        <c:crossAx val="-1537117440"/>
-        <c:crosses val="autoZero"/>
-        <c:crossBetween val="between"/>
-      </c:valAx>
-      <c:spPr>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:effectLst/>
-      </c:spPr>
-    </c:plotArea>
-    <c:legend>
-      <c:legendPos val="r"/>
-      <c:layout>
-        <c:manualLayout>
-          <c:xMode val="edge"/>
-          <c:yMode val="edge"/>
-          <c:x val="0.84085846466741432"/>
-          <c:y val="0.44849825132060006"/>
-          <c:w val="0.14382759965111558"/>
-          <c:h val="0.22512743211884409"/>
-        </c:manualLayout>
-      </c:layout>
-      <c:overlay val="0"/>
-      <c:spPr>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:effectLst/>
-      </c:spPr>
-      <c:txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr>
-            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="65000"/>
-                  <a:lumOff val="35000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:pPr>
-          <a:endParaRPr lang="en-US"/>
-        </a:p>
-      </c:txPr>
-    </c:legend>
-    <c:plotVisOnly val="1"/>
-    <c:dispBlanksAs val="gap"/>
-    <c:showDLblsOverMax val="0"/>
-  </c:chart>
-  <c:spPr>
-    <a:solidFill>
-      <a:schemeClr val="bg1"/>
-    </a:solidFill>
-    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-      <a:solidFill>
-        <a:schemeClr val="tx1">
-          <a:lumMod val="15000"/>
-          <a:lumOff val="85000"/>
-        </a:schemeClr>
-      </a:solidFill>
-      <a:round/>
-    </a:ln>
-    <a:effectLst/>
-  </c:spPr>
-  <c:txPr>
-    <a:bodyPr/>
-    <a:lstStyle/>
-    <a:p>
-      <a:pPr>
-        <a:defRPr/>
-      </a:pPr>
-      <a:endParaRPr lang="en-US"/>
-    </a:p>
-  </c:txPr>
-  <c:printSettings>
-    <c:headerFooter/>
-    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
-    <c:pageSetup/>
-  </c:printSettings>
-  <c:extLst>
-    <c:ext xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" uri="{781A3756-C4B2-4CAC-9D66-4F8BD8637D16}">
-      <c14:pivotOptions>
-        <c14:dropZoneFilter val="1"/>
-        <c14:dropZoneCategories val="1"/>
-        <c14:dropZoneData val="1"/>
-        <c14:dropZoneSeries val="1"/>
-      </c14:pivotOptions>
-    </c:ext>
-  </c:extLst>
-</c:chartSpace>
-</file>
-
-<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <c:date1904 val="0"/>
-  <c:lang val="en-US"/>
-  <c:roundedCorners val="0"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
-      <c14:style val="102"/>
-    </mc:Choice>
-    <mc:Fallback>
-      <c:style val="2"/>
-    </mc:Fallback>
-  </mc:AlternateContent>
-  <c:pivotSource>
-    <c:name>[Operations Data Validation Dashboard.xlsx]Operations Data Analysis!PivotTable1</c:name>
+    <c:name>[Operations Data Validation Dashboard.xlsx]Operations Data Analysis!PT_StatusByDepartment</c:name>
     <c:fmtId val="20"/>
   </c:pivotSource>
   <c:chart>
@@ -3119,7 +3086,7 @@
 </c:chartSpace>
 </file>
 
-<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <c:date1904 val="0"/>
   <c:lang val="en-US"/>
@@ -3133,7 +3100,7 @@
     </mc:Fallback>
   </mc:AlternateContent>
   <c:pivotSource>
-    <c:name>[Operations Data Validation Dashboard.xlsx]Operations Data Analysis!PivotTable2</c:name>
+    <c:name>[Operations Data Validation Dashboard.xlsx]Operations Data Analysis!PT_MonthlyOperations</c:name>
     <c:fmtId val="3"/>
   </c:pivotSource>
   <c:chart>
@@ -3157,11 +3124,19 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:rPr lang="en-IN" b="1"/>
+              <a:rPr lang="en-IN" b="1">
+                <a:solidFill>
+                  <a:sysClr val="windowText" lastClr="000000"/>
+                </a:solidFill>
+              </a:rPr>
               <a:t>Monthly</a:t>
             </a:r>
             <a:r>
-              <a:rPr lang="en-IN" b="1" baseline="0"/>
+              <a:rPr lang="en-IN" b="1" baseline="0">
+                <a:solidFill>
+                  <a:sysClr val="windowText" lastClr="000000"/>
+                </a:solidFill>
+              </a:rPr>
               <a:t> Operations Trends</a:t>
             </a:r>
           </a:p>
@@ -3616,7 +3591,7 @@
 </c:chartSpace>
 </file>
 
-<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <c:date1904 val="0"/>
   <c:lang val="en-US"/>
@@ -3630,7 +3605,7 @@
     </mc:Fallback>
   </mc:AlternateContent>
   <c:pivotSource>
-    <c:name>[Operations Data Validation Dashboard.xlsx]Operations Data Analysis!PivotTable3</c:name>
+    <c:name>[Operations Data Validation Dashboard.xlsx]Operations Data Analysis!PT_OperationsByFacility</c:name>
     <c:fmtId val="4"/>
   </c:pivotSource>
   <c:chart>
@@ -3654,7 +3629,11 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:rPr lang="en-IN" sz="1400" b="1" i="0" u="none" strike="noStrike" baseline="0"/>
+              <a:rPr lang="en-IN" sz="1400" b="1" i="0" u="none" strike="noStrike" baseline="0">
+                <a:solidFill>
+                  <a:sysClr val="windowText" lastClr="000000"/>
+                </a:solidFill>
+              </a:rPr>
               <a:t>Operations by Facility</a:t>
             </a:r>
           </a:p>
@@ -4096,7 +4075,7 @@
 </c:chartSpace>
 </file>
 
-<file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <c:date1904 val="0"/>
   <c:lang val="en-US"/>
@@ -4110,7 +4089,7 @@
     </mc:Fallback>
   </mc:AlternateContent>
   <c:pivotSource>
-    <c:name>[Operations Data Validation Dashboard.xlsx]Operations Data Analysis!PivotTable4</c:name>
+    <c:name>[Operations Data Validation Dashboard.xlsx]Operations Data Analysis!PT_QuantityByProcess</c:name>
     <c:fmtId val="7"/>
   </c:pivotSource>
   <c:chart>
@@ -4134,14 +4113,26 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:rPr lang="en-US"/>
+              <a:rPr lang="en-US" b="1">
+                <a:solidFill>
+                  <a:sysClr val="windowText" lastClr="000000"/>
+                </a:solidFill>
+              </a:rPr>
               <a:t>Quantity</a:t>
             </a:r>
             <a:r>
-              <a:rPr lang="en-US" baseline="0"/>
+              <a:rPr lang="en-US" b="1" baseline="0">
+                <a:solidFill>
+                  <a:sysClr val="windowText" lastClr="000000"/>
+                </a:solidFill>
+              </a:rPr>
               <a:t> by Process Type</a:t>
             </a:r>
-            <a:endParaRPr lang="en-US"/>
+            <a:endParaRPr lang="en-US" b="1">
+              <a:solidFill>
+                <a:sysClr val="windowText" lastClr="000000"/>
+              </a:solidFill>
+            </a:endParaRPr>
           </a:p>
         </c:rich>
       </c:tx>
@@ -4629,46 +4620,6 @@
 </file>
 
 <file path=xl/charts/colors4.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
-  <a:schemeClr val="accent1"/>
-  <a:schemeClr val="accent2"/>
-  <a:schemeClr val="accent3"/>
-  <a:schemeClr val="accent4"/>
-  <a:schemeClr val="accent5"/>
-  <a:schemeClr val="accent6"/>
-  <cs:variation/>
-  <cs:variation>
-    <a:lumMod val="60000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="80000"/>
-    <a:lumOff val="20000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="80000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="60000"/>
-    <a:lumOff val="40000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="50000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="70000"/>
-    <a:lumOff val="30000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="70000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="50000"/>
-    <a:lumOff val="50000"/>
-  </cs:variation>
-</cs:colorStyle>
-</file>
-
-<file path=xl/charts/colors5.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
   <a:schemeClr val="accent2"/>
@@ -5212,7 +5163,7 @@
 </file>
 
 <file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="201">
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="227">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
     <cs:fillRef idx="0"/>
@@ -5320,6 +5271,11 @@
     <cs:fontRef idx="minor">
       <a:schemeClr val="tx1"/>
     </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
   </cs:dataPoint>
   <cs:dataPoint3D>
     <cs:lnRef idx="0"/>
@@ -5330,6 +5286,11 @@
     <cs:fontRef idx="minor">
       <a:schemeClr val="tx1"/>
     </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
   </cs:dataPoint3D>
   <cs:dataPointLine>
     <cs:lnRef idx="0">
@@ -5361,6 +5322,9 @@
       <a:schemeClr val="tx1"/>
     </cs:fontRef>
     <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
       <a:ln w="9525">
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -5715,7 +5679,7 @@
 </file>
 
 <file path=xl/charts/style3.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="227">
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="201">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
     <cs:fillRef idx="0"/>
@@ -5823,11 +5787,6 @@
     <cs:fontRef idx="minor">
       <a:schemeClr val="tx1"/>
     </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="phClr"/>
-      </a:solidFill>
-    </cs:spPr>
   </cs:dataPoint>
   <cs:dataPoint3D>
     <cs:lnRef idx="0"/>
@@ -5838,11 +5797,6 @@
     <cs:fontRef idx="minor">
       <a:schemeClr val="tx1"/>
     </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="phClr"/>
-      </a:solidFill>
-    </cs:spPr>
   </cs:dataPoint3D>
   <cs:dataPointLine>
     <cs:lnRef idx="0">
@@ -5874,9 +5828,6 @@
       <a:schemeClr val="tx1"/>
     </cs:fontRef>
     <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="phClr"/>
-      </a:solidFill>
       <a:ln w="9525">
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -6733,545 +6684,7 @@
 </cs:chartStyle>
 </file>
 
-<file path=xl/charts/style5.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="201">
-  <cs:axisTitle>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="1000" kern="1200"/>
-  </cs:axisTitle>
-  <cs:categoryAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:categoryAxis>
-  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="bg1"/>
-      </a:solidFill>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="1000" kern="1200"/>
-  </cs:chartArea>
-  <cs:dataLabel>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="75000"/>
-        <a:lumOff val="25000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:dataLabel>
-  <cs:dataLabelCallout>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="lt1"/>
-      </a:solidFill>
-      <a:ln>
-        <a:solidFill>
-          <a:schemeClr val="dk1">
-            <a:lumMod val="25000"/>
-            <a:lumOff val="75000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
-      <a:spAutoFit/>
-    </cs:bodyPr>
-  </cs:dataLabelCallout>
-  <cs:dataPoint>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="1">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:dataPoint>
-  <cs:dataPoint3D>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="1">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:dataPoint3D>
-  <cs:dataPointLine>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="1"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="28575" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointLine>
-  <cs:dataPointMarker>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="1">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointMarker>
-  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
-  <cs:dataPointWireframe>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="1"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointWireframe>
-  <cs:dataTable>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:noFill/>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:dataTable>
-  <cs:downBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="dk1">
-          <a:lumMod val="65000"/>
-          <a:lumOff val="35000"/>
-        </a:schemeClr>
-      </a:solidFill>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="65000"/>
-            <a:lumOff val="35000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:downBar>
-  <cs:dropLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dropLine>
-  <cs:errorBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="65000"/>
-            <a:lumOff val="35000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:errorBar>
-  <cs:floor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:noFill/>
-      <a:ln>
-        <a:noFill/>
-      </a:ln>
-    </cs:spPr>
-  </cs:floor>
-  <cs:gridlineMajor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:gridlineMajor>
-  <cs:gridlineMinor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="5000"/>
-            <a:lumOff val="95000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:gridlineMinor>
-  <cs:hiLoLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="75000"/>
-            <a:lumOff val="25000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:hiLoLine>
-  <cs:leaderLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:leaderLine>
-  <cs:legend>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:legend>
-  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:plotArea>
-  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:plotArea3D>
-  <cs:seriesAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:seriesAxis>
-  <cs:seriesLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:seriesLine>
-  <cs:title>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
-  </cs:title>
-  <cs:trendline>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="19050" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:prstDash val="sysDot"/>
-      </a:ln>
-    </cs:spPr>
-  </cs:trendline>
-  <cs:trendlineLabel>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:trendlineLabel>
-  <cs:upBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="lt1"/>
-      </a:solidFill>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:upBar>
-  <cs:valueAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:valueAxis>
-  <cs:wall>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:noFill/>
-      <a:ln>
-        <a:noFill/>
-      </a:ln>
-    </cs:spPr>
-  </cs:wall>
-</cs:chartStyle>
-</file>
-
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>487680</xdr:colOff>
-      <xdr:row>35</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>91440</xdr:colOff>
-      <xdr:row>48</xdr:row>
-      <xdr:rowOff>53340</xdr:rowOff>
-    </xdr:to>
-    <xdr:graphicFrame macro="">
-      <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="5" name="Operations Status by Department"/>
-        <xdr:cNvGraphicFramePr/>
-      </xdr:nvGraphicFramePr>
-      <xdr:xfrm>
-        <a:off x="0" y="0"/>
-        <a:ext cx="0" cy="0"/>
-      </xdr:xfrm>
-      <a:graphic>
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-        </a:graphicData>
-      </a:graphic>
-    </xdr:graphicFrame>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
@@ -7308,13 +6721,13 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>4</xdr:col>
-      <xdr:colOff>624840</xdr:colOff>
+      <xdr:colOff>0</xdr:colOff>
       <xdr:row>5</xdr:row>
       <xdr:rowOff>175260</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>8</xdr:col>
-      <xdr:colOff>883920</xdr:colOff>
+      <xdr:colOff>15240</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>114300</xdr:rowOff>
     </xdr:to>
@@ -7345,9 +6758,9 @@
       <xdr:rowOff>7620</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>1455420</xdr:colOff>
-      <xdr:row>39</xdr:row>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>982980</xdr:colOff>
+      <xdr:row>40</xdr:row>
       <xdr:rowOff>7620</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -7378,7 +6791,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>8</xdr:col>
-      <xdr:colOff>266700</xdr:colOff>
+      <xdr:colOff>22860</xdr:colOff>
       <xdr:row>39</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
@@ -9914,7 +9327,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="PivotTable4" cacheId="9" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="5" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="5" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="8" rowHeaderCaption="Process Type">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="PT_QuantityByProcess" cacheId="9" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="5" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="5" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="8" rowHeaderCaption="Process Type">
   <location ref="D12:E18" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="11">
     <pivotField showAll="0"/>
@@ -9986,23 +9399,23 @@
     <dataField name="Sum of Quantity" fld="6" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="5">
-    <format dxfId="21">
+    <format dxfId="104">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="19">
+    <format dxfId="102">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
-    <format dxfId="17">
+    <format dxfId="100">
       <pivotArea field="4" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="15">
+    <format dxfId="98">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="4" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="13">
+    <format dxfId="96">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
   </formats>
@@ -10036,7 +9449,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="PivotTable3" cacheId="9" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="5" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="5" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="8" rowHeaderCaption="Facility">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="PT_OperationsByFacility" cacheId="9" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="5" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="5" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="8" rowHeaderCaption="Facility">
   <location ref="A24:B32" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="11">
     <pivotField dataField="1" showAll="0"/>
@@ -10098,42 +9511,33 @@
     <dataField name="Count of Operation ID" fld="0" subtotal="count" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="7">
-    <format dxfId="71">
+    <format dxfId="154">
       <pivotArea field="2" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="70">
+    <format dxfId="153">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="2" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="69">
+    <format dxfId="152">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="62">
+    <format dxfId="145">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="61">
+    <format dxfId="144">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
-    <format dxfId="55">
+    <format dxfId="138">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="54">
+    <format dxfId="137">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
   </formats>
-  <chartFormats count="2">
-    <chartFormat chart="2" format="0" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
+  <chartFormats count="1">
     <chartFormat chart="4" format="2" series="1">
       <pivotArea type="data" outline="0" fieldPosition="0">
         <references count="1">
@@ -10154,7 +9558,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="PivotTable2" cacheId="9" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="5" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="5" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="6" rowHeaderCaption="Request Date">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="PT_MonthlyOperations" cacheId="9" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="5" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="5" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="6" rowHeaderCaption="Request Date">
   <location ref="A12:B21" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="11">
     <pivotField dataField="1" showAll="0"/>
@@ -10233,25 +9637,25 @@
     <dataField name="Count of Operation ID" fld="0" subtotal="count" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="35">
-    <format dxfId="72">
+    <format dxfId="155">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="73">
+    <format dxfId="156">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
-    <format dxfId="74">
+    <format dxfId="157">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="75">
+    <format dxfId="158">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="76">
+    <format dxfId="159">
       <pivotArea field="10" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="77">
+    <format dxfId="160">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
-    <format dxfId="78">
+    <format dxfId="161">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="10" count="1">
@@ -10260,10 +9664,10 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="79">
+    <format dxfId="162">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="80">
+    <format dxfId="163">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="8" count="7">
@@ -10281,10 +9685,10 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="81">
+    <format dxfId="164">
       <pivotArea field="10" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="82">
+    <format dxfId="165">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="10" count="1">
@@ -10293,10 +9697,10 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="83">
+    <format dxfId="166">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="84">
+    <format dxfId="167">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="8" count="7">
@@ -10314,10 +9718,10 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="68">
+    <format dxfId="151">
       <pivotArea field="10" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="67">
+    <format dxfId="150">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="10" count="1">
@@ -10326,10 +9730,10 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="66">
+    <format dxfId="149">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="65">
+    <format dxfId="148">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="8" count="7">
@@ -10347,31 +9751,31 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="60">
+    <format dxfId="143">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="59">
+    <format dxfId="142">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
-    <format dxfId="53">
+    <format dxfId="136">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="52">
+    <format dxfId="135">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
-    <format dxfId="36">
+    <format dxfId="119">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="35">
+    <format dxfId="118">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="34">
+    <format dxfId="117">
       <pivotArea field="10" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="33">
+    <format dxfId="116">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
-    <format dxfId="32">
+    <format dxfId="115">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="10" count="1">
@@ -10380,10 +9784,10 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="31">
+    <format dxfId="114">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="30">
+    <format dxfId="113">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="8" count="7">
@@ -10401,19 +9805,19 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="29">
+    <format dxfId="112">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="28">
+    <format dxfId="111">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="27">
+    <format dxfId="110">
       <pivotArea field="10" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="26">
+    <format dxfId="109">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
-    <format dxfId="25">
+    <format dxfId="108">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="10" count="1">
@@ -10422,10 +9826,10 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="24">
+    <format dxfId="107">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="23">
+    <format dxfId="106">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="8" count="7">
@@ -10465,7 +9869,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="PivotTable1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="5" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="5" indent="0" compact="0" compactData="0" multipleFieldFilters="0" chartFormat="25" rowHeaderCaption="Department" colHeaderCaption="Status">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="PT_StatusByDepartment" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="5" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="5" indent="0" compact="0" compactData="0" multipleFieldFilters="0" chartFormat="29" rowHeaderCaption="Department" colHeaderCaption="Status">
   <location ref="A3:E9" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="10">
     <pivotField dataField="1" compact="0" outline="0" showAll="0" defaultSubtotal="0"/>
@@ -10535,37 +9939,37 @@
     <dataField name="Count of Operation ID" fld="0" subtotal="count" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="36">
-    <format dxfId="99">
+    <format dxfId="182">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="98">
+    <format dxfId="181">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="3" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="97">
+    <format dxfId="180">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="96">
+    <format dxfId="179">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="7" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="95">
+    <format dxfId="178">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="3" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="94">
+    <format dxfId="177">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="93">
+    <format dxfId="176">
       <pivotArea outline="0" fieldPosition="0">
         <references count="1">
           <reference field="7" count="1" selected="0">
@@ -10574,10 +9978,10 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="92">
+    <format dxfId="175">
       <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="91">
+    <format dxfId="174">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="7" count="1">
@@ -10586,7 +9990,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="90">
+    <format dxfId="173">
       <pivotArea outline="0" fieldPosition="0">
         <references count="1">
           <reference field="7" count="1" selected="0">
@@ -10595,10 +9999,10 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="89">
+    <format dxfId="172">
       <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="88">
+    <format dxfId="171">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="7" count="1">
@@ -10607,7 +10011,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="87">
+    <format dxfId="170">
       <pivotArea outline="0" fieldPosition="0">
         <references count="1">
           <reference field="7" count="1" selected="0">
@@ -10616,7 +10020,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="86">
+    <format dxfId="169">
       <pivotArea outline="0" fieldPosition="0">
         <references count="1">
           <reference field="7" count="1" selected="0">
@@ -10625,20 +10029,20 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="85">
+    <format dxfId="168">
       <pivotArea grandCol="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="64">
+    <format dxfId="147">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="3" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="63">
+    <format dxfId="146">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="58">
+    <format dxfId="141">
       <pivotArea outline="0" fieldPosition="0">
         <references count="1">
           <reference field="7" count="1" selected="0">
@@ -10647,10 +10051,10 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="57">
+    <format dxfId="140">
       <pivotArea field="7" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="56">
+    <format dxfId="139">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="7" count="1">
@@ -10659,7 +10063,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="51">
+    <format dxfId="134">
       <pivotArea outline="0" fieldPosition="0">
         <references count="1">
           <reference field="7" count="1" selected="0">
@@ -10668,10 +10072,10 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="50">
+    <format dxfId="133">
       <pivotArea field="7" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="49">
+    <format dxfId="132">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="7" count="1">
@@ -10680,59 +10084,59 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="48">
+    <format dxfId="131">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="47">
+    <format dxfId="130">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="46">
+    <format dxfId="129">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="3" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="45">
+    <format dxfId="128">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="44">
+    <format dxfId="127">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="7" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="43">
+    <format dxfId="126">
       <pivotArea dataOnly="0" labelOnly="1" grandCol="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="37">
+    <format dxfId="120">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="38">
+    <format dxfId="121">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="39">
+    <format dxfId="122">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="3" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="40">
+    <format dxfId="123">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="41">
+    <format dxfId="124">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="7" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="42">
+    <format dxfId="125">
       <pivotArea dataOnly="0" labelOnly="1" grandCol="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="11">
+    <format dxfId="94">
       <pivotArea grandCol="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
   </formats>
@@ -16270,7 +15674,7 @@
         <v>OK</v>
       </c>
       <c r="S81" s="1" t="str">
-        <f t="shared" si="4"/>
+        <f>IF(AND(L81="OK",M81="OK",N81="OK",O81="OK",P81="OK",Q81="OK",R81="OK"),"OK","REVIEW")</f>
         <v>OK</v>
       </c>
     </row>
@@ -16914,7 +16318,7 @@
   <sheetData>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B3" t="s">
         <v>153</v>
@@ -16983,38 +16387,38 @@
     <col min="3" max="3" width="10.21875" style="2" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="18.77734375" style="2" customWidth="1"/>
     <col min="5" max="5" width="14.88671875" style="2" customWidth="1"/>
-    <col min="8" max="8" width="19.5546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="22.109375" style="2" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="8.88671875" style="2"/>
   </cols>
   <sheetData>
     <row r="3" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A3" s="17" t="s">
+      <c r="A3" s="16" t="s">
         <v>147</v>
       </c>
-      <c r="B3" s="17" t="s">
+      <c r="B3" s="16" t="s">
         <v>54</v>
       </c>
-      <c r="C3" s="18"/>
-      <c r="D3" s="18"/>
-      <c r="E3" s="20"/>
-      <c r="H3" s="9" t="s">
+      <c r="C3" s="17"/>
+      <c r="D3" s="17"/>
+      <c r="E3" s="19"/>
+      <c r="H3" s="8" t="s">
         <v>141</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A4" s="17" t="s">
+      <c r="A4" s="16" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="18" t="s">
+      <c r="B4" s="17" t="s">
         <v>58</v>
       </c>
-      <c r="C4" s="18" t="s">
+      <c r="C4" s="17" t="s">
         <v>87</v>
       </c>
-      <c r="D4" s="18" t="s">
+      <c r="D4" s="17" t="s">
         <v>140</v>
       </c>
-      <c r="E4" s="20" t="s">
+      <c r="E4" s="19" t="s">
         <v>139</v>
       </c>
       <c r="H4" s="2" t="s">
@@ -17026,19 +16430,19 @@
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A5" s="18" t="s">
+      <c r="A5" s="17" t="s">
         <v>32</v>
       </c>
-      <c r="B5" s="19">
+      <c r="B5" s="18">
         <v>6</v>
       </c>
-      <c r="C5" s="19">
+      <c r="C5" s="18">
         <v>2</v>
       </c>
-      <c r="D5" s="19">
+      <c r="D5" s="18">
         <v>1</v>
       </c>
-      <c r="E5" s="21">
+      <c r="E5" s="20">
         <v>9</v>
       </c>
       <c r="H5" s="2" t="s">
@@ -17050,19 +16454,19 @@
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A6" s="18" t="s">
+      <c r="A6" s="17" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="19">
+      <c r="B6" s="18">
         <v>26</v>
       </c>
-      <c r="C6" s="19">
+      <c r="C6" s="18">
         <v>1</v>
       </c>
-      <c r="D6" s="19">
+      <c r="D6" s="18">
         <v>2</v>
       </c>
-      <c r="E6" s="21">
+      <c r="E6" s="20">
         <v>29</v>
       </c>
       <c r="H6" s="2" t="s">
@@ -17074,19 +16478,19 @@
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A7" s="18" t="s">
+      <c r="A7" s="17" t="s">
         <v>13</v>
       </c>
-      <c r="B7" s="19">
+      <c r="B7" s="18">
         <v>15</v>
       </c>
-      <c r="C7" s="19">
+      <c r="C7" s="18">
         <v>2</v>
       </c>
-      <c r="D7" s="19">
+      <c r="D7" s="18">
         <v>5</v>
       </c>
-      <c r="E7" s="21">
+      <c r="E7" s="20">
         <v>22</v>
       </c>
       <c r="H7" s="2" t="s">
@@ -17098,165 +16502,180 @@
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A8" s="18" t="s">
+      <c r="A8" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="B8" s="19">
+      <c r="B8" s="18">
         <v>18</v>
       </c>
-      <c r="C8" s="19">
+      <c r="C8" s="18">
         <v>2</v>
       </c>
-      <c r="D8" s="19"/>
-      <c r="E8" s="21">
+      <c r="D8" s="18"/>
+      <c r="E8" s="20">
         <v>20</v>
       </c>
       <c r="H8" s="2" t="s">
         <v>145</v>
       </c>
-      <c r="I8" s="8">
+      <c r="I8" s="7">
         <f>I5/I4</f>
         <v>0.8125</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A9" s="18" t="s">
+      <c r="A9" s="17" t="s">
         <v>139</v>
       </c>
-      <c r="B9" s="19">
+      <c r="B9" s="18">
         <v>65</v>
       </c>
-      <c r="C9" s="19">
+      <c r="C9" s="18">
         <v>7</v>
       </c>
-      <c r="D9" s="19">
+      <c r="D9" s="18">
         <v>8</v>
       </c>
-      <c r="E9" s="21">
+      <c r="E9" s="20">
         <v>80</v>
+      </c>
+      <c r="H9" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="I9" s="2">
+        <v>8924</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="H10" t="s">
+        <v>172</v>
+      </c>
+      <c r="I10" s="2">
+        <f>8924/80</f>
+        <v>111.55</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A12" s="17" t="s">
+      <c r="A12" s="16" t="s">
         <v>55</v>
       </c>
-      <c r="B12" s="23" t="s">
+      <c r="B12" s="22" t="s">
         <v>147</v>
       </c>
-      <c r="D12" s="14" t="s">
+      <c r="D12" s="13" t="s">
         <v>3</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A13" s="18" t="s">
-        <v>162</v>
-      </c>
-      <c r="B13" s="24"/>
+      <c r="A13" s="17" t="s">
+        <v>161</v>
+      </c>
+      <c r="B13" s="23"/>
       <c r="D13" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="E13" s="15">
+      <c r="E13" s="14">
         <v>155</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A14" s="22" t="s">
-        <v>163</v>
-      </c>
-      <c r="B14" s="24">
+      <c r="A14" s="21" t="s">
+        <v>162</v>
+      </c>
+      <c r="B14" s="23">
         <v>11</v>
       </c>
       <c r="D14" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="E14" s="15">
+      <c r="E14" s="14">
         <v>2425</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A15" s="22" t="s">
-        <v>164</v>
-      </c>
-      <c r="B15" s="24">
+      <c r="A15" s="21" t="s">
+        <v>163</v>
+      </c>
+      <c r="B15" s="23">
         <v>11</v>
       </c>
       <c r="D15" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="E15" s="15">
+      <c r="E15" s="14">
         <v>3205</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A16" s="22" t="s">
-        <v>165</v>
-      </c>
-      <c r="B16" s="24">
+      <c r="A16" s="21" t="s">
+        <v>164</v>
+      </c>
+      <c r="B16" s="23">
         <v>12</v>
       </c>
       <c r="D16" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="E16" s="15">
+      <c r="E16" s="14">
         <v>2197</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A17" s="22" t="s">
-        <v>166</v>
-      </c>
-      <c r="B17" s="24">
+      <c r="A17" s="21" t="s">
+        <v>165</v>
+      </c>
+      <c r="B17" s="23">
         <v>11</v>
       </c>
       <c r="D17" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="E17" s="15">
+      <c r="E17" s="14">
         <v>942</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A18" s="22" t="s">
-        <v>167</v>
-      </c>
-      <c r="B18" s="24">
+      <c r="A18" s="21" t="s">
+        <v>166</v>
+      </c>
+      <c r="B18" s="23">
         <v>12</v>
       </c>
       <c r="D18" s="1" t="s">
         <v>139</v>
       </c>
-      <c r="E18" s="15">
+      <c r="E18" s="14">
         <v>8924</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A19" s="22" t="s">
-        <v>168</v>
-      </c>
-      <c r="B19" s="24">
+      <c r="A19" s="21" t="s">
+        <v>167</v>
+      </c>
+      <c r="B19" s="23">
         <v>12</v>
       </c>
       <c r="D19"/>
       <c r="E19"/>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A20" s="22" t="s">
-        <v>169</v>
-      </c>
-      <c r="B20" s="24">
+      <c r="A20" s="21" t="s">
+        <v>168</v>
+      </c>
+      <c r="B20" s="23">
         <v>11</v>
       </c>
       <c r="D20"/>
       <c r="E20"/>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A21" s="18" t="s">
+      <c r="A21" s="17" t="s">
         <v>139</v>
       </c>
-      <c r="B21" s="24">
+      <c r="B21" s="23">
         <v>80</v>
       </c>
       <c r="D21"/>
@@ -17271,7 +16690,7 @@
       <c r="E23"/>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A24" s="14" t="s">
+      <c r="A24" s="13" t="s">
         <v>1</v>
       </c>
       <c r="B24" s="2" t="s">
@@ -17285,7 +16704,7 @@
       <c r="A25" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B25" s="16">
+      <c r="B25" s="15">
         <v>13</v>
       </c>
       <c r="C25"/>
@@ -17296,7 +16715,7 @@
       <c r="A26" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="B26" s="16">
+      <c r="B26" s="15">
         <v>9</v>
       </c>
       <c r="C26"/>
@@ -17307,7 +16726,7 @@
       <c r="A27" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B27" s="16">
+      <c r="B27" s="15">
         <v>9</v>
       </c>
       <c r="C27"/>
@@ -17318,7 +16737,7 @@
       <c r="A28" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="B28" s="16">
+      <c r="B28" s="15">
         <v>10</v>
       </c>
       <c r="C28"/>
@@ -17329,7 +16748,7 @@
       <c r="A29" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B29" s="16">
+      <c r="B29" s="15">
         <v>13</v>
       </c>
       <c r="C29"/>
@@ -17340,7 +16759,7 @@
       <c r="A30" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="B30" s="16">
+      <c r="B30" s="15">
         <v>14</v>
       </c>
       <c r="C30"/>
@@ -17351,7 +16770,7 @@
       <c r="A31" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="B31" s="16">
+      <c r="B31" s="15">
         <v>12</v>
       </c>
       <c r="C31"/>
@@ -17362,7 +16781,7 @@
       <c r="A32" s="1" t="s">
         <v>139</v>
       </c>
-      <c r="B32" s="16">
+      <c r="B32" s="15">
         <v>80</v>
       </c>
       <c r="C32"/>
@@ -17474,69 +16893,85 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId5"/>
-  <drawing r:id="rId6"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="5" width="22.77734375" customWidth="1"/>
-    <col min="7" max="7" width="19.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="25.77734375" customWidth="1"/>
+    <col min="3" max="4" width="25.6640625" customWidth="1"/>
+    <col min="5" max="6" width="25.77734375" customWidth="1"/>
+    <col min="7" max="7" width="25.6640625" style="2" customWidth="1"/>
+    <col min="8" max="8" width="12.6640625" customWidth="1"/>
     <col min="9" max="9" width="14.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="25.2" x14ac:dyDescent="0.3">
-      <c r="A1" s="13" t="s">
+    <row r="1" spans="1:7" ht="25.2" x14ac:dyDescent="0.3">
+      <c r="A1" s="12" t="s">
+        <v>170</v>
+      </c>
+      <c r="B1" s="12"/>
+      <c r="C1" s="12"/>
+      <c r="D1" s="12"/>
+      <c r="E1" s="12"/>
+      <c r="F1" s="12"/>
+      <c r="G1" s="12"/>
+    </row>
+    <row r="3" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A3" s="11" t="s">
+        <v>142</v>
+      </c>
+      <c r="B3" s="11" t="s">
+        <v>143</v>
+      </c>
+      <c r="C3" s="11" t="s">
+        <v>148</v>
+      </c>
+      <c r="D3" s="11" t="s">
+        <v>144</v>
+      </c>
+      <c r="E3" s="24" t="s">
+        <v>145</v>
+      </c>
+      <c r="F3" s="25" t="s">
         <v>171</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
-      <c r="F1" s="7"/>
+      <c r="G3" s="26" t="s">
+        <v>172</v>
+      </c>
     </row>
-    <row r="3" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A3" s="12" t="s">
-        <v>142</v>
-      </c>
-      <c r="B3" s="12" t="s">
-        <v>143</v>
-      </c>
-      <c r="C3" s="12" t="s">
-        <v>148</v>
-      </c>
-      <c r="D3" s="12" t="s">
-        <v>144</v>
-      </c>
-      <c r="E3" s="12" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" ht="23.4" x14ac:dyDescent="0.3">
-      <c r="A4" s="10">
+    <row r="4" spans="1:7" ht="23.4" x14ac:dyDescent="0.3">
+      <c r="A4" s="9">
         <v>80</v>
       </c>
-      <c r="B4" s="10">
+      <c r="B4" s="9">
         <v>65</v>
       </c>
-      <c r="C4" s="10">
+      <c r="C4" s="9">
         <v>7</v>
       </c>
-      <c r="D4" s="10">
+      <c r="D4" s="9">
         <v>8</v>
       </c>
-      <c r="E4" s="11">
+      <c r="E4" s="10">
         <v>0.8125</v>
+      </c>
+      <c r="F4" s="9">
+        <v>8924</v>
+      </c>
+      <c r="G4" s="9">
+        <v>111.5</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A1:G1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>